<commit_message>
Fixed a small bug in partnership targets
</commit_message>
<xml_diff>
--- a/input/partnered_share_targets.xlsx
+++ b/input/partnered_share_targets.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/SimPathsUK_refactored/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://essexuniversity-my.sharepoint.com/personal/mv25449_essex_ac_uk/Documents/WorkCEMPA/SimPathsUK/validate_alignments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBCF1CCB-1C3E-3747-A1C0-2097BA55A002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_B35981270C6F3FCBB6307EF3E0442AF071040EA2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69195529-DB8A-304D-B795-0FB6A9697688}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="30240" windowHeight="19640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="partnered_share" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -422,7 +422,7 @@
         <v>2011</v>
       </c>
       <c r="B2" s="2">
-        <v>0.63057139662305717</v>
+        <v>0.64881080389022827</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -430,7 +430,7 @@
         <v>2012</v>
       </c>
       <c r="B3" s="2">
-        <v>0.62911308623298035</v>
+        <v>0.64325892925262451</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -438,7 +438,7 @@
         <v>2013</v>
       </c>
       <c r="B4" s="2">
-        <v>0.6244072872473172</v>
+        <v>0.63569384813308716</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -446,7 +446,7 @@
         <v>2014</v>
       </c>
       <c r="B5" s="2">
-        <v>0.62604367373153502</v>
+        <v>0.63734567165374756</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -454,7 +454,7 @@
         <v>2015</v>
       </c>
       <c r="B6" s="2">
-        <v>0.62868757259001162</v>
+        <v>0.64118802547454834</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -462,7 +462,7 @@
         <v>2016</v>
       </c>
       <c r="B7" s="2">
-        <v>0.62058932772068842</v>
+        <v>0.63751119375228882</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -470,7 +470,7 @@
         <v>2017</v>
       </c>
       <c r="B8" s="2">
-        <v>0.61782259724223088</v>
+        <v>0.64006215333938599</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -478,7 +478,7 @@
         <v>2018</v>
       </c>
       <c r="B9" s="2">
-        <v>0.61249863671065552</v>
+        <v>0.63119488954544067</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -486,7 +486,7 @@
         <v>2019</v>
       </c>
       <c r="B10" s="2">
-        <v>0.61124121779859486</v>
+        <v>0.63247203826904297</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -494,7 +494,7 @@
         <v>2020</v>
       </c>
       <c r="B11" s="2">
-        <v>0.60652290438296297</v>
+        <v>0.62348079681396484</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -502,7 +502,7 @@
         <v>2021</v>
       </c>
       <c r="B12" s="2">
-        <v>0.60516042180839125</v>
+        <v>0.63103306293487549</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -510,7 +510,7 @@
         <v>2022</v>
       </c>
       <c r="B13" s="2">
-        <v>0.60333794534763063</v>
+        <v>0.61048740148544312</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -518,7 +518,7 @@
         <v>2023</v>
       </c>
       <c r="B14" s="2">
-        <v>0.58993023961176827</v>
+        <v>0.58404338359832764</v>
       </c>
     </row>
   </sheetData>

</xml_diff>